<commit_message>
Dashboard edit: AVL in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -571,7 +571,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>70000.0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>https://app.smartsheet.com/sheets/FgQPXjG9HQg2M4vfH2jpcgvmjMC22HQV29VQwh31?view=grid</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>

</xml_diff>

<commit_message>
Dashboard edit: SSPM in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -22,10 +22,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -72,7 +72,7 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -569,10 +569,8 @@
       <c r="C2" s="2" t="n">
         <v>47696</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>70000</t>
-        </is>
+      <c r="D2" t="n">
+        <v>70000</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -594,7 +592,7 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="b">
+      <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -615,7 +613,7 @@
           <t>Azure/CloudBerry (NC)</t>
         </is>
       </c>
-      <c r="R2" t="b">
+      <c r="R2" t="n">
         <v>1</v>
       </c>
       <c r="S2" t="inlineStr">
@@ -625,7 +623,7 @@
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
-      <c r="V2" t="b">
+      <c r="V2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -640,7 +638,7 @@
           <t>Christensen, O'Connor, Johnson, Kindness</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>46554</v>
       </c>
       <c r="D3" t="n">
@@ -665,13 +663,13 @@
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="3" t="n">
+      <c r="J3" s="2" t="n">
         <v>46044</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" s="3" t="n">
+      <c r="L3" s="2" t="n">
         <v>46044</v>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -712,7 +710,7 @@
           <t>City of Covina</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>46965</v>
       </c>
       <c r="D4" t="n">
@@ -741,13 +739,13 @@
           <t>July- June</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" s="2" t="n">
         <v>46070</v>
       </c>
       <c r="K4" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="3" t="n">
+      <c r="L4" s="2" t="n">
         <v>46072</v>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -799,13 +797,13 @@
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="3" t="n">
+      <c r="J5" s="2" t="n">
         <v>46038</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="3" t="n">
+      <c r="L5" s="2" t="n">
         <v>46042</v>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -846,7 +844,7 @@
           <t>City of Duvall</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>46074</v>
       </c>
       <c r="D6" t="n">
@@ -906,7 +904,7 @@
           <t>City of Goleta</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="2" t="n">
         <v>46568</v>
       </c>
       <c r="D7" t="n">
@@ -935,13 +933,13 @@
           <t>July-June</t>
         </is>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="J7" s="2" t="n">
         <v>46043</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="3" t="n">
+      <c r="L7" s="2" t="n">
         <v>46044</v>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -978,7 +976,7 @@
           <t>City of Industry</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="2" t="n">
         <v>46326</v>
       </c>
       <c r="D8" t="n">
@@ -1046,7 +1044,7 @@
           <t>City of Monrovia</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="2" t="n">
         <v>47664</v>
       </c>
       <c r="D9" t="n">
@@ -1071,13 +1069,13 @@
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="3" t="n">
+      <c r="J9" s="2" t="n">
         <v>46077</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="3" t="n">
+      <c r="L9" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1114,7 +1112,7 @@
           <t>City of Ranchos Palos Verdes</t>
         </is>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="2" t="n">
         <v>46559</v>
       </c>
       <c r="D10" t="n">
@@ -1178,7 +1176,7 @@
           <t>City of San Fernando</t>
         </is>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="2" t="n">
         <v>46326</v>
       </c>
       <c r="D11" t="n">
@@ -1238,7 +1236,7 @@
           <t>SmartStop Asset Management</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="2" t="n">
         <v>46630</v>
       </c>
       <c r="D12" t="n">
@@ -1313,8 +1311,10 @@
       <c r="C13" s="3" t="n">
         <v>46630</v>
       </c>
-      <c r="D13" t="n">
-        <v>35030</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>35030.0</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="n">
+      <c r="K13" t="b">
         <v>0</v>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1349,15 +1349,19 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="n">
+      <c r="R13" t="b">
         <v>1</v>
       </c>
-      <c r="S13" t="n">
-        <v>1</v>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/38WGJ4QMm4WmHgPfm3V6pMMPV5Cxh9qvrvPGfrG1?view=grid</t>
+        </is>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
+      <c r="V13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1370,7 +1374,7 @@
           <t>SmartStop REIT</t>
         </is>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="2" t="n">
         <v>46630</v>
       </c>
       <c r="D14" t="n">
@@ -1428,7 +1432,7 @@
           <t>Sunnylands</t>
         </is>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="D15" t="n">
@@ -1457,13 +1461,13 @@
           <t>July-June</t>
         </is>
       </c>
-      <c r="J15" s="3" t="n">
+      <c r="J15" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" s="3" t="n">
+      <c r="L15" s="2" t="n">
         <v>46052</v>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1504,7 +1508,7 @@
           <t>Desert Water Agency</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="2" t="n">
         <v>45530</v>
       </c>
       <c r="D16" t="n">
@@ -1529,13 +1533,13 @@
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="3" t="n">
+      <c r="J16" s="2" t="n">
         <v>46083</v>
       </c>
       <c r="K16" t="n">
         <v>1</v>
       </c>
-      <c r="L16" s="3" t="n">
+      <c r="L16" s="2" t="n">
         <v>46085</v>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -1572,7 +1576,7 @@
           <t>Adams Campbell Construction</t>
         </is>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="2" t="n">
         <v>46419</v>
       </c>
       <c r="D17" t="n">
@@ -1636,7 +1640,7 @@
           <t>Adhoc Labs</t>
         </is>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="2" t="n">
         <v>46157</v>
       </c>
       <c r="D18" t="n">
@@ -1696,7 +1700,7 @@
           <t>Baghouse</t>
         </is>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="D19" t="n">
@@ -1760,7 +1764,7 @@
           <t>Boys and Girls Club of Redlands</t>
         </is>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="D20" t="n">
@@ -1789,7 +1793,7 @@
           <t>July- June</t>
         </is>
       </c>
-      <c r="J20" s="3" t="n">
+      <c r="J20" s="2" t="n">
         <v>46070</v>
       </c>
       <c r="K20" t="n">
@@ -1892,7 +1896,7 @@
           <t>Central Basin Municipal Water District</t>
         </is>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C22" s="2" t="n">
         <v>47483</v>
       </c>
       <c r="D22" t="n">
@@ -1922,7 +1926,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="inlineStr"/>
-      <c r="M22" s="3" t="n">
+      <c r="M22" s="2" t="n">
         <v>46104</v>
       </c>
       <c r="N22" t="inlineStr"/>
@@ -1954,7 +1958,7 @@
           <t>CMSD</t>
         </is>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C23" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="D23" t="n">
@@ -1979,14 +1983,14 @@
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="3" t="n">
+      <c r="J23" s="2" t="n">
         <v>46085</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
       </c>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" s="3" t="n">
+      <c r="M23" s="2" t="n">
         <v>46104</v>
       </c>
       <c r="N23" t="inlineStr"/>
@@ -2018,7 +2022,7 @@
           <t>Hesperia Recreation and Park District</t>
         </is>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C24" s="2" t="n">
         <v>45303</v>
       </c>
       <c r="D24" t="n">
@@ -2082,7 +2086,7 @@
           <t>LeVecke Corporation</t>
         </is>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C25" s="2" t="n">
         <v>46752</v>
       </c>
       <c r="D25" t="n">
@@ -2146,7 +2150,7 @@
           <t>Pacific Railway Enterprises, Inc.</t>
         </is>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C26" s="2" t="n">
         <v>46177</v>
       </c>
       <c r="D26" t="n">
@@ -2241,13 +2245,13 @@
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" s="3" t="n">
+      <c r="J27" s="2" t="n">
         <v>46065</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
       </c>
-      <c r="L27" s="3" t="n">
+      <c r="L27" s="2" t="n">
         <v>46070</v>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -2284,7 +2288,7 @@
           <t>Rubidoux Community Services District</t>
         </is>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C28" s="2" t="n">
         <v>45991</v>
       </c>
       <c r="D28" t="n">
@@ -2317,7 +2321,7 @@
       <c r="K28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" s="3" t="n">
+      <c r="L28" s="2" t="n">
         <v>46042</v>
       </c>
       <c r="M28" t="inlineStr"/>
@@ -2358,7 +2362,7 @@
           <t>Superior Court of California Nevada</t>
         </is>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C29" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="D29" t="n">
@@ -2414,7 +2418,7 @@
           <t>SolarMax</t>
         </is>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" s="2" t="n">
         <v>46446</v>
       </c>
       <c r="D30" t="n">
@@ -2482,7 +2486,7 @@
           <t>TruEvolution</t>
         </is>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C31" s="2" t="n">
         <v>46813</v>
       </c>
       <c r="D31" t="n">
@@ -2542,7 +2546,7 @@
           <t>AAA Paving Co.</t>
         </is>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C32" s="2" t="n">
         <v>46446</v>
       </c>
       <c r="D32" t="n">
@@ -2567,7 +2571,7 @@
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="3" t="n">
+      <c r="J32" s="2" t="n">
         <v>46072</v>
       </c>
       <c r="K32" t="n">
@@ -2608,7 +2612,7 @@
           <t>A1 Grit</t>
         </is>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C33" s="2" t="n">
         <v>44936</v>
       </c>
       <c r="D33" t="n">
@@ -2664,7 +2668,7 @@
           <t>Alpine Water Users Association</t>
         </is>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C34" s="2" t="n">
         <v>46388</v>
       </c>
       <c r="D34" t="n">
@@ -2720,7 +2724,7 @@
           <t>Beaumont Cherry Valley Recreation &amp; Park District</t>
         </is>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C35" s="2" t="n">
         <v>45563</v>
       </c>
       <c r="D35" t="n">
@@ -2834,7 +2838,7 @@
           <t>Continental Recycling</t>
         </is>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C37" s="2" t="n">
         <v>46477</v>
       </c>
       <c r="D37" t="n">
@@ -2890,7 +2894,7 @@
           <t>Discovery Eye Foundation</t>
         </is>
       </c>
-      <c r="C38" s="3" t="n">
+      <c r="C38" s="2" t="n">
         <v>46446</v>
       </c>
       <c r="D38" t="n">
@@ -2915,7 +2919,7 @@
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="3" t="n">
+      <c r="J38" s="2" t="n">
         <v>46072</v>
       </c>
       <c r="K38" t="n">
@@ -2948,7 +2952,7 @@
           <t>Dobler Law Group</t>
         </is>
       </c>
-      <c r="C39" s="3" t="n">
+      <c r="C39" s="2" t="n">
         <v>45839</v>
       </c>
       <c r="D39" t="n">
@@ -3031,13 +3035,13 @@
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="3" t="n">
+      <c r="J40" s="2" t="n">
         <v>46076</v>
       </c>
       <c r="K40" t="n">
         <v>1</v>
       </c>
-      <c r="L40" s="3" t="n">
+      <c r="L40" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="M40" t="inlineStr"/>
@@ -3066,7 +3070,7 @@
           <t>Genesis Supreme &amp; PCW</t>
         </is>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="C41" s="2" t="n">
         <v>46903</v>
       </c>
       <c r="D41" t="n">
@@ -3095,7 +3099,7 @@
       <c r="K41" t="n">
         <v>0</v>
       </c>
-      <c r="L41" s="3" t="n">
+      <c r="L41" s="2" t="n">
         <v>45945</v>
       </c>
       <c r="M41" t="inlineStr"/>
@@ -3232,7 +3236,7 @@
           <t>Larry Jacinto Construction</t>
         </is>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="C44" s="2" t="n">
         <v>46387</v>
       </c>
       <c r="D44" t="n">
@@ -3261,7 +3265,7 @@
       <c r="K44" t="n">
         <v>0</v>
       </c>
-      <c r="L44" s="3" t="n">
+      <c r="L44" s="2" t="n">
         <v>46044</v>
       </c>
       <c r="M44" t="inlineStr"/>
@@ -3290,7 +3294,7 @@
           <t>Lift to Rise</t>
         </is>
       </c>
-      <c r="C45" s="3" t="n">
+      <c r="C45" s="2" t="n">
         <v>45748</v>
       </c>
       <c r="D45" t="n">
@@ -3346,7 +3350,7 @@
           <t>Loma Linda University</t>
         </is>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="C46" s="2" t="n">
         <v>46904</v>
       </c>
       <c r="D46" t="n">
@@ -3375,16 +3379,16 @@
           <t>July - June</t>
         </is>
       </c>
-      <c r="J46" s="3" t="n">
+      <c r="J46" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="K46" t="n">
         <v>1</v>
       </c>
-      <c r="L46" s="3" t="n">
+      <c r="L46" s="2" t="n">
         <v>46078</v>
       </c>
-      <c r="M46" s="3" t="n">
+      <c r="M46" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="N46" t="inlineStr"/>
@@ -3470,7 +3474,7 @@
           <t>Open Gym Partner</t>
         </is>
       </c>
-      <c r="C48" s="3" t="n">
+      <c r="C48" s="2" t="n">
         <v>46538</v>
       </c>
       <c r="D48" t="n">
@@ -3526,7 +3530,7 @@
           <t>Riverside County Childcare Consortium</t>
         </is>
       </c>
-      <c r="C49" s="3" t="n">
+      <c r="C49" s="2" t="n">
         <v>46811</v>
       </c>
       <c r="D49" t="n">
@@ -3582,7 +3586,7 @@
           <t>Industry Business Council</t>
         </is>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="C50" s="2" t="n">
         <v>46965</v>
       </c>
       <c r="D50" t="n">
@@ -4855,7 +4859,7 @@
           <t>Avalon Transportation</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="2" t="n">
         <v>47696</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -4890,7 +4894,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M6" s="3" t="n">
+      <c r="M6" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N6" t="inlineStr"/>
@@ -4909,7 +4913,7 @@
           <t>Christensen, O'Connor, Johnson, Kindness</t>
         </is>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="2" t="n">
         <v>46554</v>
       </c>
       <c r="E7" t="inlineStr">
@@ -4944,7 +4948,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M7" s="3" t="n">
+      <c r="M7" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N7" t="inlineStr"/>
@@ -4963,7 +4967,7 @@
           <t>City of Covina</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="2" t="n">
         <v>46965</v>
       </c>
       <c r="E8" t="inlineStr">
@@ -4998,7 +5002,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M8" s="3" t="n">
+      <c r="M8" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N8" t="inlineStr"/>
@@ -5050,7 +5054,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M9" s="3" t="n">
+      <c r="M9" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N9" t="inlineStr"/>
@@ -5069,7 +5073,7 @@
           <t>City of Goleta</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="2" t="n">
         <v>46568</v>
       </c>
       <c r="E10" t="inlineStr">
@@ -5104,7 +5108,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M10" s="3" t="n">
+      <c r="M10" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N10" t="inlineStr"/>
@@ -5123,7 +5127,7 @@
           <t>City of Duvall</t>
         </is>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="2" t="n">
         <v>46074</v>
       </c>
       <c r="E11" t="inlineStr">
@@ -5158,7 +5162,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M11" s="3" t="n">
+      <c r="M11" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N11" t="inlineStr"/>
@@ -5177,7 +5181,7 @@
           <t>City of Industry</t>
         </is>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="2" t="n">
         <v>46326</v>
       </c>
       <c r="E12" t="inlineStr">
@@ -5212,7 +5216,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M12" s="3" t="n">
+      <c r="M12" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N12" t="inlineStr"/>
@@ -5262,7 +5266,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M13" s="3" t="n">
+      <c r="M13" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N13" t="inlineStr"/>
@@ -5281,7 +5285,7 @@
           <t>City of Monrovia</t>
         </is>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="2" t="n">
         <v>47664</v>
       </c>
       <c r="E14" t="inlineStr">
@@ -5316,7 +5320,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M14" s="3" t="n">
+      <c r="M14" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -5335,7 +5339,7 @@
           <t>City of Ranchos Palos Verdes</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="2" t="n">
         <v>46559</v>
       </c>
       <c r="E15" t="inlineStr">
@@ -5370,7 +5374,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M15" s="3" t="n">
+      <c r="M15" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N15" t="inlineStr"/>
@@ -5389,7 +5393,7 @@
           <t>City of San Fernando</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="2" t="n">
         <v>46326</v>
       </c>
       <c r="E16" t="inlineStr">
@@ -5424,7 +5428,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M16" s="3" t="n">
+      <c r="M16" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N16" t="inlineStr"/>
@@ -5443,7 +5447,7 @@
           <t>City of South Pasadena &amp; Police Department</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="2" t="n">
         <v>46022</v>
       </c>
       <c r="E17" t="inlineStr">
@@ -5466,7 +5470,7 @@
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
-      <c r="M17" s="3" t="n">
+      <c r="M17" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N17" t="inlineStr">
@@ -5489,7 +5493,7 @@
           <t>Desert Water Agency</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="2" t="n">
         <v>45530</v>
       </c>
       <c r="E18" t="inlineStr">
@@ -5516,7 +5520,7 @@
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
-      <c r="M18" s="3" t="n">
+      <c r="M18" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N18" t="inlineStr"/>
@@ -5535,7 +5539,7 @@
           <t>SmartStop Asset Management</t>
         </is>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="2" t="n">
         <v>46630</v>
       </c>
       <c r="E19" t="inlineStr">
@@ -5570,7 +5574,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M19" s="3" t="n">
+      <c r="M19" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N19" t="inlineStr"/>
@@ -5589,7 +5593,7 @@
           <t>SmartStop Property Management</t>
         </is>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="2" t="n">
         <v>46630</v>
       </c>
       <c r="E20" t="inlineStr">
@@ -5620,7 +5624,7 @@
           <t>Budget Reviewed Already</t>
         </is>
       </c>
-      <c r="M20" s="3" t="n">
+      <c r="M20" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N20" t="inlineStr"/>
@@ -5639,7 +5643,7 @@
           <t>SmartStop REIT</t>
         </is>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="2" t="n">
         <v>46630</v>
       </c>
       <c r="E21" t="inlineStr">
@@ -5674,7 +5678,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M21" s="3" t="n">
+      <c r="M21" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N21" t="inlineStr"/>
@@ -5693,7 +5697,7 @@
           <t>Sunnylands</t>
         </is>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="E22" t="inlineStr">
@@ -5728,7 +5732,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M22" s="3" t="n">
+      <c r="M22" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N22" t="inlineStr"/>
@@ -5747,7 +5751,7 @@
           <t>Adams Campbell Construction</t>
         </is>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="2" t="n">
         <v>46419</v>
       </c>
       <c r="E23" t="inlineStr">
@@ -5770,7 +5774,7 @@
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" s="3" t="n">
+      <c r="M23" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N23" t="inlineStr">
@@ -5793,7 +5797,7 @@
           <t>Adhoc Labs</t>
         </is>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="2" t="n">
         <v>46157</v>
       </c>
       <c r="E24" t="inlineStr">
@@ -5828,7 +5832,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M24" s="3" t="n">
+      <c r="M24" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N24" t="inlineStr"/>
@@ -5847,7 +5851,7 @@
           <t>Baghouse</t>
         </is>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="E25" t="inlineStr">
@@ -5882,7 +5886,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M25" s="3" t="n">
+      <c r="M25" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N25" t="inlineStr"/>
@@ -5917,7 +5921,7 @@
           <t>Boys and Girls Club of Redlands</t>
         </is>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="E27" t="inlineStr">
@@ -5952,7 +5956,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M27" s="3" t="n">
+      <c r="M27" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N27" t="inlineStr"/>
@@ -6008,7 +6012,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M28" s="3" t="n">
+      <c r="M28" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N28" t="inlineStr"/>
@@ -6027,7 +6031,7 @@
           <t>Central Basin Municipal Water District</t>
         </is>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" s="2" t="n">
         <v>47483</v>
       </c>
       <c r="E29" t="inlineStr">
@@ -6062,7 +6066,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M29" s="3" t="n">
+      <c r="M29" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N29" t="inlineStr"/>
@@ -6081,7 +6085,7 @@
           <t>Costa Mesa Sanitary District</t>
         </is>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D30" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="E30" t="inlineStr">
@@ -6116,7 +6120,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M30" s="3" t="n">
+      <c r="M30" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N30" t="inlineStr"/>
@@ -6135,7 +6139,7 @@
           <t>Hesperia Recreation and Park District</t>
         </is>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D31" s="2" t="n">
         <v>45303</v>
       </c>
       <c r="E31" t="inlineStr">
@@ -6170,7 +6174,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M31" s="3" t="n">
+      <c r="M31" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N31" t="inlineStr"/>
@@ -6189,7 +6193,7 @@
           <t>LeVecke Corporation</t>
         </is>
       </c>
-      <c r="D32" s="3" t="n">
+      <c r="D32" s="2" t="n">
         <v>46752</v>
       </c>
       <c r="E32" t="inlineStr">
@@ -6224,7 +6228,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M32" s="3" t="n">
+      <c r="M32" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N32" t="inlineStr"/>
@@ -6243,7 +6247,7 @@
           <t>Pacific Railway Enterprises, Inc.</t>
         </is>
       </c>
-      <c r="D33" s="3" t="n">
+      <c r="D33" s="2" t="n">
         <v>46177</v>
       </c>
       <c r="E33" t="inlineStr">
@@ -6278,7 +6282,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M33" s="3" t="n">
+      <c r="M33" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N33" t="inlineStr"/>
@@ -6334,7 +6338,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M34" s="3" t="n">
+      <c r="M34" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N34" t="inlineStr"/>
@@ -6390,7 +6394,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M35" s="3" t="n">
+      <c r="M35" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N35" t="inlineStr"/>
@@ -6409,7 +6413,7 @@
           <t>Superior Court of California Nevada</t>
         </is>
       </c>
-      <c r="D36" s="3" t="n">
+      <c r="D36" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="E36" t="inlineStr">
@@ -6436,7 +6440,7 @@
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
-      <c r="M36" s="3" t="n">
+      <c r="M36" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N36" t="inlineStr">
@@ -6459,7 +6463,7 @@
           <t>SolarMax</t>
         </is>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D37" s="2" t="n">
         <v>46446</v>
       </c>
       <c r="E37" t="inlineStr">
@@ -6494,7 +6498,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M37" s="3" t="n">
+      <c r="M37" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N37" t="inlineStr"/>
@@ -6513,7 +6517,7 @@
           <t>TruEvolution</t>
         </is>
       </c>
-      <c r="D38" s="3" t="n">
+      <c r="D38" s="2" t="n">
         <v>46813</v>
       </c>
       <c r="E38" t="inlineStr">
@@ -6548,7 +6552,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M38" s="3" t="n">
+      <c r="M38" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N38" t="inlineStr"/>
@@ -6567,7 +6571,7 @@
           <t>AAA Paving Co.</t>
         </is>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D39" s="2" t="n">
         <v>46446</v>
       </c>
       <c r="E39" t="inlineStr">
@@ -6602,7 +6606,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M39" s="3" t="n">
+      <c r="M39" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N39" t="inlineStr"/>
@@ -6621,7 +6625,7 @@
           <t>A1 Grit</t>
         </is>
       </c>
-      <c r="D40" s="3" t="n">
+      <c r="D40" s="2" t="n">
         <v>44936</v>
       </c>
       <c r="E40" t="inlineStr">
@@ -6656,7 +6660,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M40" s="3" t="n">
+      <c r="M40" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N40" t="inlineStr"/>
@@ -6675,7 +6679,7 @@
           <t>Beaumont Cherry Valley Recreation &amp; Park District</t>
         </is>
       </c>
-      <c r="D41" s="3" t="n">
+      <c r="D41" s="2" t="n">
         <v>45563</v>
       </c>
       <c r="E41" t="inlineStr">
@@ -6710,7 +6714,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M41" s="3" t="n">
+      <c r="M41" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N41" t="inlineStr"/>
@@ -6729,7 +6733,7 @@
           <t>Alpine Water Users Association</t>
         </is>
       </c>
-      <c r="D42" s="3" t="n">
+      <c r="D42" s="2" t="n">
         <v>46388</v>
       </c>
       <c r="E42" t="inlineStr">
@@ -6764,7 +6768,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M42" s="3" t="n">
+      <c r="M42" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N42" t="inlineStr"/>
@@ -6820,7 +6824,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M43" s="3" t="n">
+      <c r="M43" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N43" t="inlineStr"/>
@@ -6839,7 +6843,7 @@
           <t>Continental Recycling</t>
         </is>
       </c>
-      <c r="D44" s="3" t="n">
+      <c r="D44" s="2" t="n">
         <v>46477</v>
       </c>
       <c r="E44" t="inlineStr">
@@ -6874,7 +6878,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M44" s="3" t="n">
+      <c r="M44" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N44" t="inlineStr"/>
@@ -6893,7 +6897,7 @@
           <t>Discovery Eye Foundation</t>
         </is>
       </c>
-      <c r="D45" s="3" t="n">
+      <c r="D45" s="2" t="n">
         <v>46446</v>
       </c>
       <c r="E45" t="inlineStr">
@@ -6928,7 +6932,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M45" s="3" t="n">
+      <c r="M45" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N45" t="inlineStr"/>
@@ -6963,7 +6967,7 @@
           <t>Dobler Law Group</t>
         </is>
       </c>
-      <c r="D47" s="3" t="n">
+      <c r="D47" s="2" t="n">
         <v>45839</v>
       </c>
       <c r="E47" t="inlineStr">
@@ -6998,7 +7002,7 @@
           <t>Offboarding Phase</t>
         </is>
       </c>
-      <c r="M47" s="3" t="n">
+      <c r="M47" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N47" t="inlineStr"/>
@@ -7054,7 +7058,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M48" s="3" t="n">
+      <c r="M48" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N48" t="inlineStr"/>
@@ -7073,7 +7077,7 @@
           <t>Genesis Supreme &amp; PCW</t>
         </is>
       </c>
-      <c r="D49" s="3" t="n">
+      <c r="D49" s="2" t="n">
         <v>46903</v>
       </c>
       <c r="E49" t="inlineStr">
@@ -7108,7 +7112,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M49" s="3" t="n">
+      <c r="M49" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N49" t="inlineStr"/>
@@ -7164,7 +7168,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M50" s="3" t="n">
+      <c r="M50" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N50" t="inlineStr"/>
@@ -7200,7 +7204,7 @@
       </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
-      <c r="M51" s="3" t="n">
+      <c r="M51" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N51" t="inlineStr"/>
@@ -7219,7 +7223,7 @@
           <t>Larry Jacinto Construction</t>
         </is>
       </c>
-      <c r="D52" s="3" t="n">
+      <c r="D52" s="2" t="n">
         <v>46387</v>
       </c>
       <c r="E52" t="inlineStr">
@@ -7254,7 +7258,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M52" s="3" t="n">
+      <c r="M52" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N52" t="inlineStr"/>
@@ -7273,7 +7277,7 @@
           <t>Lift to Rise</t>
         </is>
       </c>
-      <c r="D53" s="3" t="n">
+      <c r="D53" s="2" t="n">
         <v>45748</v>
       </c>
       <c r="E53" t="inlineStr">
@@ -7308,7 +7312,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M53" s="3" t="n">
+      <c r="M53" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N53" t="inlineStr"/>
@@ -7327,7 +7331,7 @@
           <t>Loma Linda University</t>
         </is>
       </c>
-      <c r="D54" s="3" t="n">
+      <c r="D54" s="2" t="n">
         <v>46904</v>
       </c>
       <c r="E54" t="inlineStr">
@@ -7362,7 +7366,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M54" s="3" t="n">
+      <c r="M54" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N54" t="inlineStr"/>
@@ -7410,7 +7414,7 @@
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
-      <c r="M55" s="3" t="n">
+      <c r="M55" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N55" t="inlineStr"/>
@@ -7429,7 +7433,7 @@
           <t>Open Gym Partner</t>
         </is>
       </c>
-      <c r="D56" s="3" t="n">
+      <c r="D56" s="2" t="n">
         <v>46538</v>
       </c>
       <c r="E56" t="inlineStr">
@@ -7464,7 +7468,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M56" s="3" t="n">
+      <c r="M56" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N56" t="inlineStr"/>
@@ -7483,7 +7487,7 @@
           <t>Riverside County Childcare Consortium</t>
         </is>
       </c>
-      <c r="D57" s="3" t="n">
+      <c r="D57" s="2" t="n">
         <v>46811</v>
       </c>
       <c r="E57" t="inlineStr">
@@ -7518,7 +7522,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M57" s="3" t="n">
+      <c r="M57" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N57" t="inlineStr"/>
@@ -7537,7 +7541,7 @@
           <t>Industry Business Council</t>
         </is>
       </c>
-      <c r="D58" s="3" t="n">
+      <c r="D58" s="2" t="n">
         <v>46965</v>
       </c>
       <c r="E58" t="inlineStr">
@@ -7572,7 +7576,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M58" s="3" t="n">
+      <c r="M58" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N58" t="inlineStr"/>
@@ -7640,7 +7644,7 @@
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
-      <c r="M61" s="3" t="n">
+      <c r="M61" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="N61" t="inlineStr"/>
@@ -7765,7 +7769,7 @@
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" s="3" t="n">
+      <c r="L4" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7791,7 +7795,7 @@
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" s="3" t="n">
+      <c r="L5" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7817,7 +7821,7 @@
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" s="3" t="n">
+      <c r="L6" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7843,7 +7847,7 @@
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" s="3" t="n">
+      <c r="L7" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7869,7 +7873,7 @@
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" s="3" t="n">
+      <c r="L8" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7895,7 +7899,7 @@
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" s="3" t="n">
+      <c r="L9" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7953,7 +7957,7 @@
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" s="3" t="n">
+      <c r="L12" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7979,7 +7983,7 @@
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" s="3" t="n">
+      <c r="L13" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8005,7 +8009,7 @@
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" s="3" t="n">
+      <c r="L14" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8023,7 +8027,7 @@
           <t>Lester &amp; Cantrell</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="2" t="n">
         <v>46387</v>
       </c>
       <c r="E15" t="n">
@@ -8039,7 +8043,7 @@
         </is>
       </c>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" s="3" t="n">
+      <c r="L15" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8095,7 +8099,7 @@
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" s="3" t="n">
+      <c r="L18" s="2" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8119,7 +8123,7 @@
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" s="3" t="n">
+      <c r="L19" s="2" t="n">
         <v>46006</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard edit: SSR in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -1308,13 +1308,11 @@
           <t>SmartStop Property Management</t>
         </is>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="2" t="n">
         <v>46630</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>35030.0</t>
-        </is>
+      <c r="D13" t="n">
+        <v>35030</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1340,7 +1338,7 @@
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="b">
+      <c r="K13" t="n">
         <v>0</v>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1349,7 +1347,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="b">
+      <c r="R13" t="n">
         <v>1</v>
       </c>
       <c r="S13" t="inlineStr">
@@ -1359,7 +1357,7 @@
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
-      <c r="V13" t="b">
+      <c r="V13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1374,11 +1372,13 @@
           <t>SmartStop REIT</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="3" t="n">
         <v>46630</v>
       </c>
-      <c r="D14" t="n">
-        <v>38860</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>38860.0</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="n">
+      <c r="K14" t="b">
         <v>0</v>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -1413,13 +1413,19 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="n">
+      <c r="R14" t="b">
         <v>1</v>
       </c>
-      <c r="S14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/38WGJ4QMm4WmHgPfm3V6pMMPV5Cxh9qvrvPGfrG1?view=grid</t>
+        </is>
+      </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
+      <c r="V14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: AL in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -1372,13 +1372,11 @@
           <t>SmartStop REIT</t>
         </is>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="2" t="n">
         <v>46630</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>38860.0</t>
-        </is>
+      <c r="D14" t="n">
+        <v>38860</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1404,7 +1402,7 @@
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="b">
+      <c r="K14" t="n">
         <v>0</v>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -1413,7 +1411,7 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="b">
+      <c r="R14" t="n">
         <v>1</v>
       </c>
       <c r="S14" t="inlineStr">
@@ -1423,7 +1421,7 @@
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
-      <c r="V14" t="b">
+      <c r="V14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1646,11 +1644,13 @@
           <t>Adhoc Labs</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="3" t="n">
         <v>46157</v>
       </c>
-      <c r="D18" t="n">
-        <v>4017.5</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4017.5</t>
+        </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="n">
+      <c r="K18" t="b">
         <v>0</v>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -1685,15 +1685,19 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="n">
+      <c r="R18" t="b">
         <v>1</v>
       </c>
-      <c r="S18" t="n">
-        <v>1</v>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/FXmc8P8PR9qgCpPG58jM484XGVcjJPcp7j82w2h1?view=grid</t>
+        </is>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
+      <c r="V18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: CBMWD in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -1644,13 +1644,11 @@
           <t>Adhoc Labs</t>
         </is>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="2" t="n">
         <v>46157</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>4017.5</t>
-        </is>
+      <c r="D18" t="n">
+        <v>4017.5</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1676,7 +1674,7 @@
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="b">
+      <c r="K18" t="n">
         <v>0</v>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -1685,7 +1683,7 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="b">
+      <c r="R18" t="n">
         <v>1</v>
       </c>
       <c r="S18" t="inlineStr">
@@ -1695,7 +1693,7 @@
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
-      <c r="V18" t="b">
+      <c r="V18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1906,11 +1904,13 @@
           <t>Central Basin Municipal Water District</t>
         </is>
       </c>
-      <c r="C22" s="2" t="n">
+      <c r="C22" s="3" t="n">
         <v>47483</v>
       </c>
-      <c r="D22" t="n">
-        <v>7000</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>7000.0</t>
+        </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="n">
+      <c r="K22" t="b">
         <v>0</v>
       </c>
       <c r="L22" t="inlineStr"/>
@@ -1947,15 +1947,19 @@
       </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="n">
+      <c r="R22" t="b">
         <v>1</v>
       </c>
-      <c r="S22" t="n">
-        <v>1</v>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/rpc4qHFxW3hF9cHGfVvgqF8X557WqPwqp97Qp971?view=grid</t>
+        </is>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
+      <c r="V22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: SOLAR in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -1904,13 +1904,11 @@
           <t>Central Basin Municipal Water District</t>
         </is>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C22" s="2" t="n">
         <v>47483</v>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>7000.0</t>
-        </is>
+      <c r="D22" t="n">
+        <v>7000</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1932,7 +1930,7 @@
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="b">
+      <c r="K22" t="n">
         <v>0</v>
       </c>
       <c r="L22" t="inlineStr"/>
@@ -1947,7 +1945,7 @@
       </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="b">
+      <c r="R22" t="n">
         <v>1</v>
       </c>
       <c r="S22" t="inlineStr">
@@ -1957,7 +1955,7 @@
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
-      <c r="V22" t="b">
+      <c r="V22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2432,11 +2430,13 @@
           <t>SolarMax</t>
         </is>
       </c>
-      <c r="C30" s="2" t="n">
+      <c r="C30" s="3" t="n">
         <v>46446</v>
       </c>
-      <c r="D30" t="n">
-        <v>6650</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>6650.0</t>
+        </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="n">
+      <c r="K30" t="b">
         <v>0</v>
       </c>
       <c r="L30" t="inlineStr"/>
@@ -2479,15 +2479,19 @@
           <t>Local Backup (CB)</t>
         </is>
       </c>
-      <c r="R30" t="n">
+      <c r="R30" t="b">
         <v>1</v>
       </c>
-      <c r="S30" t="n">
-        <v>1</v>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/rXc87335Mr7VgJxCf58775vfWG2JRQRGCw4rwX41?view=gantt</t>
+        </is>
       </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
+      <c r="V30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: LLU in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -2430,13 +2430,11 @@
           <t>SolarMax</t>
         </is>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" s="2" t="n">
         <v>46446</v>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>6650.0</t>
-        </is>
+      <c r="D30" t="n">
+        <v>6650</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2458,7 +2456,7 @@
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="b">
+      <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" t="inlineStr"/>
@@ -2479,7 +2477,7 @@
           <t>Local Backup (CB)</t>
         </is>
       </c>
-      <c r="R30" t="b">
+      <c r="R30" t="n">
         <v>1</v>
       </c>
       <c r="S30" t="inlineStr">
@@ -2489,7 +2487,7 @@
       </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="b">
+      <c r="V30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3368,11 +3366,13 @@
           <t>Loma Linda University</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n">
+      <c r="C46" s="3" t="n">
         <v>46904</v>
       </c>
-      <c r="D46" t="n">
-        <v>1960</v>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1960.0</t>
+        </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
       <c r="J46" s="2" t="n">
         <v>46073</v>
       </c>
-      <c r="K46" t="n">
+      <c r="K46" t="b">
         <v>1</v>
       </c>
       <c r="L46" s="2" t="n">
@@ -3413,15 +3413,19 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="n">
+      <c r="R46" t="b">
         <v>1</v>
       </c>
-      <c r="S46" t="n">
-        <v>1</v>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/3J9vvQrmJhvCFw8jH3CwQXRfP4Vr3mrqCv7mmPc1?view=grid</t>
+        </is>
       </c>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
-      <c r="V46" t="inlineStr"/>
+      <c r="V46" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: LJC in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -3252,11 +3252,13 @@
           <t>Larry Jacinto Construction</t>
         </is>
       </c>
-      <c r="C44" s="2" t="n">
+      <c r="C44" s="3" t="n">
         <v>46387</v>
       </c>
-      <c r="D44" t="n">
-        <v>2100</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -3278,7 +3280,7 @@
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
-      <c r="K44" t="n">
+      <c r="K44" t="b">
         <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
@@ -3289,15 +3291,19 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="n">
+      <c r="R44" t="b">
         <v>1</v>
       </c>
-      <c r="S44" t="n">
-        <v>1</v>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/g7JppWRVfpxmjR7vrQXGhWQhW9pC42h6rc4vmqf1?view=grid</t>
+        </is>
       </c>
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
-      <c r="V44" t="inlineStr"/>
+      <c r="V44" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3366,13 +3372,11 @@
           <t>Loma Linda University</t>
         </is>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="C46" s="2" t="n">
         <v>46904</v>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>1960.0</t>
-        </is>
+      <c r="D46" t="n">
+        <v>1960</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -3400,7 +3404,7 @@
       <c r="J46" s="2" t="n">
         <v>46073</v>
       </c>
-      <c r="K46" t="b">
+      <c r="K46" t="n">
         <v>1</v>
       </c>
       <c r="L46" s="2" t="n">
@@ -3413,7 +3417,7 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="b">
+      <c r="R46" t="n">
         <v>1</v>
       </c>
       <c r="S46" t="inlineStr">
@@ -3423,7 +3427,7 @@
       </c>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
-      <c r="V46" t="b">
+      <c r="V46" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard edit: AAA in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -2562,11 +2562,13 @@
           <t>AAA Paving Co.</t>
         </is>
       </c>
-      <c r="C32" s="2" t="n">
+      <c r="C32" s="3" t="n">
         <v>46446</v>
       </c>
-      <c r="D32" t="n">
-        <v>2100</v>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2100.0</t>
+        </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2590,10 +2592,12 @@
       <c r="J32" s="2" t="n">
         <v>46072</v>
       </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="inlineStr"/>
+      <c r="K32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>46093</v>
+      </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
@@ -2607,15 +2611,19 @@
           <t>Local Backup (CB)</t>
         </is>
       </c>
-      <c r="R32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S32" t="n">
-        <v>0</v>
+      <c r="R32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
+      <c r="V32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3252,13 +3260,11 @@
           <t>Larry Jacinto Construction</t>
         </is>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="C44" s="2" t="n">
         <v>46387</v>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2100.0</t>
-        </is>
+      <c r="D44" t="n">
+        <v>2100</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -3280,7 +3286,7 @@
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
-      <c r="K44" t="b">
+      <c r="K44" t="n">
         <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
@@ -3291,7 +3297,7 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="b">
+      <c r="R44" t="n">
         <v>1</v>
       </c>
       <c r="S44" t="inlineStr">
@@ -3301,7 +3307,7 @@
       </c>
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
-      <c r="V44" t="b">
+      <c r="V44" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard edit: CMSD in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -1970,11 +1970,13 @@
           <t>CMSD</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n">
+      <c r="C23" s="3" t="n">
         <v>46203</v>
       </c>
-      <c r="D23" t="n">
-        <v>5730</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>5730.0</t>
+        </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1998,10 +2000,12 @@
       <c r="J23" s="2" t="n">
         <v>46085</v>
       </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="inlineStr"/>
+      <c r="K23" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>46097</v>
+      </c>
       <c r="M23" s="2" t="n">
         <v>46104</v>
       </c>
@@ -2013,15 +2017,19 @@
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="n">
+      <c r="R23" t="b">
         <v>1</v>
       </c>
-      <c r="S23" t="n">
-        <v>1</v>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
+      <c r="V23" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2562,13 +2570,11 @@
           <t>AAA Paving Co.</t>
         </is>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C32" s="2" t="n">
         <v>46446</v>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>2100.0</t>
-        </is>
+      <c r="D32" t="n">
+        <v>2100</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2592,7 +2598,7 @@
       <c r="J32" s="2" t="n">
         <v>46072</v>
       </c>
-      <c r="K32" t="b">
+      <c r="K32" t="n">
         <v>1</v>
       </c>
       <c r="L32" s="2" t="n">
@@ -2611,7 +2617,7 @@
           <t>Local Backup (CB)</t>
         </is>
       </c>
-      <c r="R32" t="b">
+      <c r="R32" t="n">
         <v>0</v>
       </c>
       <c r="S32" t="inlineStr">
@@ -2621,7 +2627,7 @@
       </c>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
-      <c r="V32" t="b">
+      <c r="V32" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard edit: BGCRED in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -1772,11 +1772,13 @@
           <t>Boys and Girls Club of Redlands</t>
         </is>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C20" s="3" t="n">
         <v>46203</v>
       </c>
-      <c r="D20" t="n">
-        <v>4314</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>4314.0</t>
+        </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1804,7 +1806,7 @@
       <c r="J20" s="2" t="n">
         <v>46070</v>
       </c>
-      <c r="K20" t="n">
+      <c r="K20" t="b">
         <v>0</v>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -1821,15 +1823,19 @@
           <t>NEEDS NAS URGENTLY</t>
         </is>
       </c>
-      <c r="R20" t="n">
+      <c r="R20" t="b">
         <v>1</v>
       </c>
-      <c r="S20" t="n">
-        <v>1</v>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/gMq9cqC56rXWRHr9pWm9p8v8vcxj83QpcGjVW3J1?view=grid</t>
+        </is>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
+      <c r="V20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1970,13 +1976,11 @@
           <t>CMSD</t>
         </is>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C23" s="2" t="n">
         <v>46203</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>5730.0</t>
-        </is>
+      <c r="D23" t="n">
+        <v>5730</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2000,7 +2004,7 @@
       <c r="J23" s="2" t="n">
         <v>46085</v>
       </c>
-      <c r="K23" t="b">
+      <c r="K23" t="n">
         <v>1</v>
       </c>
       <c r="L23" s="2" t="n">
@@ -2015,7 +2019,7 @@
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="b">
+      <c r="R23" t="n">
         <v>1</v>
       </c>
       <c r="S23" t="inlineStr">
@@ -2025,7 +2029,7 @@
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="b">
+      <c r="V23" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard edit: COD in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -27,16 +27,13 @@
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -47,7 +44,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -55,26 +52,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,112 +429,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Customer Code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Customer Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Contract Expiration</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>MRR</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Seats</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Contract Type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Fiscal Year</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>QBR vCIO Generated</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Signed off by C/U</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Last BR</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Next BR</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Q1 QBR Closure TARGET</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>CyberSuite?</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Firewall Equipment</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Backup (Immutable)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Pre/Check-in meetings?</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Smartsheet</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Bio/Glue/POC/IAM//New User/SteerCo update</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Contract Summary/Customer Profile</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Face time/Gift check-in</t>
         </is>
@@ -566,7 +551,7 @@
           <t>Avalon Transportation</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="1" t="n">
         <v>47696</v>
       </c>
       <c r="D2" t="n">
@@ -638,7 +623,7 @@
           <t>Christensen, O'Connor, Johnson, Kindness</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="1" t="n">
         <v>46554</v>
       </c>
       <c r="D3" t="n">
@@ -663,13 +648,13 @@
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>46044</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="L3" s="1" t="n">
         <v>46044</v>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -710,7 +695,7 @@
           <t>City of Covina</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="1" t="n">
         <v>46965</v>
       </c>
       <c r="D4" t="n">
@@ -739,13 +724,13 @@
           <t>July- June</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>46070</v>
       </c>
       <c r="K4" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="L4" s="1" t="n">
         <v>46072</v>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -797,13 +782,13 @@
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>46038</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="L5" s="1" t="n">
         <v>46042</v>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -847,8 +832,10 @@
       <c r="C6" s="2" t="n">
         <v>46074</v>
       </c>
-      <c r="D6" t="n">
-        <v>21121</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>21121.0</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -870,7 +857,7 @@
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="n">
+      <c r="K6" t="b">
         <v>0</v>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -883,15 +870,19 @@
       </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="n">
+      <c r="R6" t="b">
         <v>1</v>
       </c>
-      <c r="S6" t="n">
-        <v>1</v>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/PVWcWHqM7jMpWgXvJWg7V6rcqgGp8pQHXQPPGXJ1?view=grid</t>
+        </is>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
+      <c r="V6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -904,7 +895,7 @@
           <t>City of Goleta</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="1" t="n">
         <v>46568</v>
       </c>
       <c r="D7" t="n">
@@ -933,13 +924,13 @@
           <t>July-June</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="2" t="n">
+      <c r="L7" s="1" t="n">
         <v>46044</v>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -976,7 +967,7 @@
           <t>City of Industry</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="1" t="n">
         <v>46326</v>
       </c>
       <c r="D8" t="n">
@@ -1044,7 +1035,7 @@
           <t>City of Monrovia</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="1" t="n">
         <v>47664</v>
       </c>
       <c r="D9" t="n">
@@ -1069,13 +1060,13 @@
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46077</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="L9" s="1" t="n">
         <v>46078</v>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1112,7 +1103,7 @@
           <t>City of Ranchos Palos Verdes</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="1" t="n">
         <v>46559</v>
       </c>
       <c r="D10" t="n">
@@ -1176,7 +1167,7 @@
           <t>City of San Fernando</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="1" t="n">
         <v>46326</v>
       </c>
       <c r="D11" t="n">
@@ -1236,7 +1227,7 @@
           <t>SmartStop Asset Management</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="1" t="n">
         <v>46630</v>
       </c>
       <c r="D12" t="n">
@@ -1308,7 +1299,7 @@
           <t>SmartStop Property Management</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" s="1" t="n">
         <v>46630</v>
       </c>
       <c r="D13" t="n">
@@ -1372,7 +1363,7 @@
           <t>SmartStop REIT</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="1" t="n">
         <v>46630</v>
       </c>
       <c r="D14" t="n">
@@ -1436,7 +1427,7 @@
           <t>Sunnylands</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C15" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="D15" t="n">
@@ -1465,13 +1456,13 @@
           <t>July-June</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" s="2" t="n">
+      <c r="L15" s="1" t="n">
         <v>46052</v>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1512,7 +1503,7 @@
           <t>Desert Water Agency</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="1" t="n">
         <v>45530</v>
       </c>
       <c r="D16" t="n">
@@ -1537,13 +1528,13 @@
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
+      <c r="J16" s="1" t="n">
         <v>46083</v>
       </c>
       <c r="K16" t="n">
         <v>1</v>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="L16" s="1" t="n">
         <v>46085</v>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -1580,7 +1571,7 @@
           <t>Adams Campbell Construction</t>
         </is>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="C17" s="1" t="n">
         <v>46419</v>
       </c>
       <c r="D17" t="n">
@@ -1644,7 +1635,7 @@
           <t>Adhoc Labs</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="1" t="n">
         <v>46157</v>
       </c>
       <c r="D18" t="n">
@@ -1708,7 +1699,7 @@
           <t>Baghouse</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C19" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="D19" t="n">
@@ -1772,13 +1763,11 @@
           <t>Boys and Girls Club of Redlands</t>
         </is>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="1" t="n">
         <v>46203</v>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>4314.0</t>
-        </is>
+      <c r="D20" t="n">
+        <v>4314</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1803,10 +1792,10 @@
           <t>July- June</t>
         </is>
       </c>
-      <c r="J20" s="2" t="n">
+      <c r="J20" s="1" t="n">
         <v>46070</v>
       </c>
-      <c r="K20" t="b">
+      <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -1823,7 +1812,7 @@
           <t>NEEDS NAS URGENTLY</t>
         </is>
       </c>
-      <c r="R20" t="b">
+      <c r="R20" t="n">
         <v>1</v>
       </c>
       <c r="S20" t="inlineStr">
@@ -1833,7 +1822,7 @@
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
-      <c r="V20" t="b">
+      <c r="V20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1910,7 +1899,7 @@
           <t>Central Basin Municipal Water District</t>
         </is>
       </c>
-      <c r="C22" s="2" t="n">
+      <c r="C22" s="1" t="n">
         <v>47483</v>
       </c>
       <c r="D22" t="n">
@@ -1940,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="inlineStr"/>
-      <c r="M22" s="2" t="n">
+      <c r="M22" s="1" t="n">
         <v>46104</v>
       </c>
       <c r="N22" t="inlineStr"/>
@@ -1976,7 +1965,7 @@
           <t>CMSD</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n">
+      <c r="C23" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="D23" t="n">
@@ -2001,13 +1990,13 @@
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
+      <c r="J23" s="1" t="n">
         <v>46085</v>
       </c>
       <c r="K23" t="n">
         <v>1</v>
       </c>
-      <c r="L23" s="2" t="n">
+      <c r="L23" s="1" t="n">
         <v>46097</v>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -2044,7 +2033,7 @@
           <t>Hesperia Recreation and Park District</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C24" s="1" t="n">
         <v>45303</v>
       </c>
       <c r="D24" t="n">
@@ -2108,7 +2097,7 @@
           <t>LeVecke Corporation</t>
         </is>
       </c>
-      <c r="C25" s="2" t="n">
+      <c r="C25" s="1" t="n">
         <v>46752</v>
       </c>
       <c r="D25" t="n">
@@ -2172,7 +2161,7 @@
           <t>Pacific Railway Enterprises, Inc.</t>
         </is>
       </c>
-      <c r="C26" s="2" t="n">
+      <c r="C26" s="1" t="n">
         <v>46177</v>
       </c>
       <c r="D26" t="n">
@@ -2267,13 +2256,13 @@
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" s="2" t="n">
+      <c r="J27" s="1" t="n">
         <v>46065</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
       </c>
-      <c r="L27" s="2" t="n">
+      <c r="L27" s="1" t="n">
         <v>46070</v>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -2310,7 +2299,7 @@
           <t>Rubidoux Community Services District</t>
         </is>
       </c>
-      <c r="C28" s="2" t="n">
+      <c r="C28" s="1" t="n">
         <v>45991</v>
       </c>
       <c r="D28" t="n">
@@ -2343,7 +2332,7 @@
       <c r="K28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" s="2" t="n">
+      <c r="L28" s="1" t="n">
         <v>46042</v>
       </c>
       <c r="M28" t="inlineStr"/>
@@ -2384,7 +2373,7 @@
           <t>Superior Court of California Nevada</t>
         </is>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C29" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="D29" t="n">
@@ -2440,7 +2429,7 @@
           <t>SolarMax</t>
         </is>
       </c>
-      <c r="C30" s="2" t="n">
+      <c r="C30" s="1" t="n">
         <v>46446</v>
       </c>
       <c r="D30" t="n">
@@ -2512,7 +2501,7 @@
           <t>TruEvolution</t>
         </is>
       </c>
-      <c r="C31" s="2" t="n">
+      <c r="C31" s="1" t="n">
         <v>46813</v>
       </c>
       <c r="D31" t="n">
@@ -2572,7 +2561,7 @@
           <t>AAA Paving Co.</t>
         </is>
       </c>
-      <c r="C32" s="2" t="n">
+      <c r="C32" s="1" t="n">
         <v>46446</v>
       </c>
       <c r="D32" t="n">
@@ -2597,13 +2586,13 @@
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="2" t="n">
+      <c r="J32" s="1" t="n">
         <v>46072</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
       </c>
-      <c r="L32" s="2" t="n">
+      <c r="L32" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="M32" t="inlineStr"/>
@@ -2644,7 +2633,7 @@
           <t>A1 Grit</t>
         </is>
       </c>
-      <c r="C33" s="2" t="n">
+      <c r="C33" s="1" t="n">
         <v>44936</v>
       </c>
       <c r="D33" t="n">
@@ -2700,7 +2689,7 @@
           <t>Alpine Water Users Association</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C34" s="1" t="n">
         <v>46388</v>
       </c>
       <c r="D34" t="n">
@@ -2756,7 +2745,7 @@
           <t>Beaumont Cherry Valley Recreation &amp; Park District</t>
         </is>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C35" s="1" t="n">
         <v>45563</v>
       </c>
       <c r="D35" t="n">
@@ -2870,7 +2859,7 @@
           <t>Continental Recycling</t>
         </is>
       </c>
-      <c r="C37" s="2" t="n">
+      <c r="C37" s="1" t="n">
         <v>46477</v>
       </c>
       <c r="D37" t="n">
@@ -2926,7 +2915,7 @@
           <t>Discovery Eye Foundation</t>
         </is>
       </c>
-      <c r="C38" s="2" t="n">
+      <c r="C38" s="1" t="n">
         <v>46446</v>
       </c>
       <c r="D38" t="n">
@@ -2951,7 +2940,7 @@
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="2" t="n">
+      <c r="J38" s="1" t="n">
         <v>46072</v>
       </c>
       <c r="K38" t="n">
@@ -2984,7 +2973,7 @@
           <t>Dobler Law Group</t>
         </is>
       </c>
-      <c r="C39" s="2" t="n">
+      <c r="C39" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="D39" t="n">
@@ -3067,13 +3056,13 @@
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="2" t="n">
+      <c r="J40" s="1" t="n">
         <v>46076</v>
       </c>
       <c r="K40" t="n">
         <v>1</v>
       </c>
-      <c r="L40" s="2" t="n">
+      <c r="L40" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="M40" t="inlineStr"/>
@@ -3102,7 +3091,7 @@
           <t>Genesis Supreme &amp; PCW</t>
         </is>
       </c>
-      <c r="C41" s="2" t="n">
+      <c r="C41" s="1" t="n">
         <v>46903</v>
       </c>
       <c r="D41" t="n">
@@ -3131,7 +3120,7 @@
       <c r="K41" t="n">
         <v>0</v>
       </c>
-      <c r="L41" s="2" t="n">
+      <c r="L41" s="1" t="n">
         <v>45945</v>
       </c>
       <c r="M41" t="inlineStr"/>
@@ -3268,7 +3257,7 @@
           <t>Larry Jacinto Construction</t>
         </is>
       </c>
-      <c r="C44" s="2" t="n">
+      <c r="C44" s="1" t="n">
         <v>46387</v>
       </c>
       <c r="D44" t="n">
@@ -3297,7 +3286,7 @@
       <c r="K44" t="n">
         <v>0</v>
       </c>
-      <c r="L44" s="2" t="n">
+      <c r="L44" s="1" t="n">
         <v>46044</v>
       </c>
       <c r="M44" t="inlineStr"/>
@@ -3330,7 +3319,7 @@
           <t>Lift to Rise</t>
         </is>
       </c>
-      <c r="C45" s="2" t="n">
+      <c r="C45" s="1" t="n">
         <v>45748</v>
       </c>
       <c r="D45" t="n">
@@ -3386,7 +3375,7 @@
           <t>Loma Linda University</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n">
+      <c r="C46" s="1" t="n">
         <v>46904</v>
       </c>
       <c r="D46" t="n">
@@ -3415,16 +3404,16 @@
           <t>July - June</t>
         </is>
       </c>
-      <c r="J46" s="2" t="n">
+      <c r="J46" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="K46" t="n">
         <v>1</v>
       </c>
-      <c r="L46" s="2" t="n">
+      <c r="L46" s="1" t="n">
         <v>46078</v>
       </c>
-      <c r="M46" s="2" t="n">
+      <c r="M46" s="1" t="n">
         <v>46078</v>
       </c>
       <c r="N46" t="inlineStr"/>
@@ -3514,7 +3503,7 @@
           <t>Open Gym Partner</t>
         </is>
       </c>
-      <c r="C48" s="2" t="n">
+      <c r="C48" s="1" t="n">
         <v>46538</v>
       </c>
       <c r="D48" t="n">
@@ -3570,7 +3559,7 @@
           <t>Riverside County Childcare Consortium</t>
         </is>
       </c>
-      <c r="C49" s="2" t="n">
+      <c r="C49" s="1" t="n">
         <v>46811</v>
       </c>
       <c r="D49" t="n">
@@ -3626,7 +3615,7 @@
           <t>Industry Business Council</t>
         </is>
       </c>
-      <c r="C50" s="2" t="n">
+      <c r="C50" s="1" t="n">
         <v>46965</v>
       </c>
       <c r="D50" t="n">
@@ -3734,22 +3723,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Customer Code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Customer Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Project Rate</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Proposed Rate</t>
         </is>
@@ -4814,72 +4803,72 @@
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Customer Code</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Customer Name</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Contract Expiration</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>MRR</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Current IT Services MRC</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Proposed IT-Services</t>
         </is>
       </c>
-      <c r="I5" s="1" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>MRC Difference</t>
         </is>
       </c>
-      <c r="J5" s="1" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Alignment report completion date</t>
         </is>
       </c>
-      <c r="K5" s="1" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Strategy Review</t>
         </is>
       </c>
-      <c r="L5" s="1" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Strategy Road Map</t>
         </is>
       </c>
-      <c r="M5" s="1" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Budget Creation</t>
         </is>
       </c>
-      <c r="N5" s="1" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -4899,7 +4888,7 @@
           <t>Avalon Transportation</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="1" t="n">
         <v>47696</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -4934,7 +4923,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="M6" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N6" t="inlineStr"/>
@@ -4953,7 +4942,7 @@
           <t>Christensen, O'Connor, Johnson, Kindness</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="1" t="n">
         <v>46554</v>
       </c>
       <c r="E7" t="inlineStr">
@@ -4988,7 +4977,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N7" t="inlineStr"/>
@@ -5007,7 +4996,7 @@
           <t>City of Covina</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="1" t="n">
         <v>46965</v>
       </c>
       <c r="E8" t="inlineStr">
@@ -5042,7 +5031,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="M8" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N8" t="inlineStr"/>
@@ -5094,7 +5083,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="M9" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N9" t="inlineStr"/>
@@ -5113,7 +5102,7 @@
           <t>City of Goleta</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="1" t="n">
         <v>46568</v>
       </c>
       <c r="E10" t="inlineStr">
@@ -5148,7 +5137,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="M10" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N10" t="inlineStr"/>
@@ -5167,7 +5156,7 @@
           <t>City of Duvall</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="1" t="n">
         <v>46074</v>
       </c>
       <c r="E11" t="inlineStr">
@@ -5202,7 +5191,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="M11" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N11" t="inlineStr"/>
@@ -5221,7 +5210,7 @@
           <t>City of Industry</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="1" t="n">
         <v>46326</v>
       </c>
       <c r="E12" t="inlineStr">
@@ -5256,7 +5245,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M12" s="2" t="n">
+      <c r="M12" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N12" t="inlineStr"/>
@@ -5306,7 +5295,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="M13" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N13" t="inlineStr"/>
@@ -5325,7 +5314,7 @@
           <t>City of Monrovia</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="1" t="n">
         <v>47664</v>
       </c>
       <c r="E14" t="inlineStr">
@@ -5360,7 +5349,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="M14" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -5379,7 +5368,7 @@
           <t>City of Ranchos Palos Verdes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="1" t="n">
         <v>46559</v>
       </c>
       <c r="E15" t="inlineStr">
@@ -5414,7 +5403,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="M15" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N15" t="inlineStr"/>
@@ -5433,7 +5422,7 @@
           <t>City of San Fernando</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="1" t="n">
         <v>46326</v>
       </c>
       <c r="E16" t="inlineStr">
@@ -5468,7 +5457,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="M16" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N16" t="inlineStr"/>
@@ -5487,7 +5476,7 @@
           <t>City of South Pasadena &amp; Police Department</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" s="1" t="n">
         <v>46022</v>
       </c>
       <c r="E17" t="inlineStr">
@@ -5510,7 +5499,7 @@
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
-      <c r="M17" s="2" t="n">
+      <c r="M17" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N17" t="inlineStr">
@@ -5533,7 +5522,7 @@
           <t>Desert Water Agency</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="1" t="n">
         <v>45530</v>
       </c>
       <c r="E18" t="inlineStr">
@@ -5560,7 +5549,7 @@
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
-      <c r="M18" s="2" t="n">
+      <c r="M18" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N18" t="inlineStr"/>
@@ -5579,7 +5568,7 @@
           <t>SmartStop Asset Management</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D19" s="1" t="n">
         <v>46630</v>
       </c>
       <c r="E19" t="inlineStr">
@@ -5614,7 +5603,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M19" s="2" t="n">
+      <c r="M19" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N19" t="inlineStr"/>
@@ -5633,7 +5622,7 @@
           <t>SmartStop Property Management</t>
         </is>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="1" t="n">
         <v>46630</v>
       </c>
       <c r="E20" t="inlineStr">
@@ -5664,7 +5653,7 @@
           <t>Budget Reviewed Already</t>
         </is>
       </c>
-      <c r="M20" s="2" t="n">
+      <c r="M20" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N20" t="inlineStr"/>
@@ -5683,7 +5672,7 @@
           <t>SmartStop REIT</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n">
+      <c r="D21" s="1" t="n">
         <v>46630</v>
       </c>
       <c r="E21" t="inlineStr">
@@ -5718,7 +5707,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M21" s="2" t="n">
+      <c r="M21" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N21" t="inlineStr"/>
@@ -5737,7 +5726,7 @@
           <t>Sunnylands</t>
         </is>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D22" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="E22" t="inlineStr">
@@ -5772,7 +5761,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M22" s="2" t="n">
+      <c r="M22" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N22" t="inlineStr"/>
@@ -5791,7 +5780,7 @@
           <t>Adams Campbell Construction</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n">
+      <c r="D23" s="1" t="n">
         <v>46419</v>
       </c>
       <c r="E23" t="inlineStr">
@@ -5814,7 +5803,7 @@
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
+      <c r="M23" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N23" t="inlineStr">
@@ -5837,7 +5826,7 @@
           <t>Adhoc Labs</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D24" s="1" t="n">
         <v>46157</v>
       </c>
       <c r="E24" t="inlineStr">
@@ -5872,7 +5861,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M24" s="2" t="n">
+      <c r="M24" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N24" t="inlineStr"/>
@@ -5891,7 +5880,7 @@
           <t>Baghouse</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n">
+      <c r="D25" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="E25" t="inlineStr">
@@ -5926,7 +5915,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M25" s="2" t="n">
+      <c r="M25" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N25" t="inlineStr"/>
@@ -5961,7 +5950,7 @@
           <t>Boys and Girls Club of Redlands</t>
         </is>
       </c>
-      <c r="D27" s="2" t="n">
+      <c r="D27" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="E27" t="inlineStr">
@@ -5996,7 +5985,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M27" s="2" t="n">
+      <c r="M27" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N27" t="inlineStr"/>
@@ -6052,7 +6041,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M28" s="2" t="n">
+      <c r="M28" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N28" t="inlineStr"/>
@@ -6071,7 +6060,7 @@
           <t>Central Basin Municipal Water District</t>
         </is>
       </c>
-      <c r="D29" s="2" t="n">
+      <c r="D29" s="1" t="n">
         <v>47483</v>
       </c>
       <c r="E29" t="inlineStr">
@@ -6106,7 +6095,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M29" s="2" t="n">
+      <c r="M29" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N29" t="inlineStr"/>
@@ -6125,7 +6114,7 @@
           <t>Costa Mesa Sanitary District</t>
         </is>
       </c>
-      <c r="D30" s="2" t="n">
+      <c r="D30" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="E30" t="inlineStr">
@@ -6160,7 +6149,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M30" s="2" t="n">
+      <c r="M30" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N30" t="inlineStr"/>
@@ -6179,7 +6168,7 @@
           <t>Hesperia Recreation and Park District</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n">
+      <c r="D31" s="1" t="n">
         <v>45303</v>
       </c>
       <c r="E31" t="inlineStr">
@@ -6214,7 +6203,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M31" s="2" t="n">
+      <c r="M31" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N31" t="inlineStr"/>
@@ -6233,7 +6222,7 @@
           <t>LeVecke Corporation</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n">
+      <c r="D32" s="1" t="n">
         <v>46752</v>
       </c>
       <c r="E32" t="inlineStr">
@@ -6268,7 +6257,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M32" s="2" t="n">
+      <c r="M32" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N32" t="inlineStr"/>
@@ -6287,7 +6276,7 @@
           <t>Pacific Railway Enterprises, Inc.</t>
         </is>
       </c>
-      <c r="D33" s="2" t="n">
+      <c r="D33" s="1" t="n">
         <v>46177</v>
       </c>
       <c r="E33" t="inlineStr">
@@ -6322,7 +6311,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M33" s="2" t="n">
+      <c r="M33" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N33" t="inlineStr"/>
@@ -6378,7 +6367,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M34" s="2" t="n">
+      <c r="M34" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N34" t="inlineStr"/>
@@ -6434,7 +6423,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M35" s="2" t="n">
+      <c r="M35" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N35" t="inlineStr"/>
@@ -6453,7 +6442,7 @@
           <t>Superior Court of California Nevada</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D36" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="E36" t="inlineStr">
@@ -6480,7 +6469,7 @@
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
-      <c r="M36" s="2" t="n">
+      <c r="M36" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N36" t="inlineStr">
@@ -6503,7 +6492,7 @@
           <t>SolarMax</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n">
+      <c r="D37" s="1" t="n">
         <v>46446</v>
       </c>
       <c r="E37" t="inlineStr">
@@ -6538,7 +6527,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M37" s="2" t="n">
+      <c r="M37" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N37" t="inlineStr"/>
@@ -6557,7 +6546,7 @@
           <t>TruEvolution</t>
         </is>
       </c>
-      <c r="D38" s="2" t="n">
+      <c r="D38" s="1" t="n">
         <v>46813</v>
       </c>
       <c r="E38" t="inlineStr">
@@ -6592,7 +6581,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M38" s="2" t="n">
+      <c r="M38" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N38" t="inlineStr"/>
@@ -6611,7 +6600,7 @@
           <t>AAA Paving Co.</t>
         </is>
       </c>
-      <c r="D39" s="2" t="n">
+      <c r="D39" s="1" t="n">
         <v>46446</v>
       </c>
       <c r="E39" t="inlineStr">
@@ -6646,7 +6635,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M39" s="2" t="n">
+      <c r="M39" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N39" t="inlineStr"/>
@@ -6665,7 +6654,7 @@
           <t>A1 Grit</t>
         </is>
       </c>
-      <c r="D40" s="2" t="n">
+      <c r="D40" s="1" t="n">
         <v>44936</v>
       </c>
       <c r="E40" t="inlineStr">
@@ -6700,7 +6689,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M40" s="2" t="n">
+      <c r="M40" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N40" t="inlineStr"/>
@@ -6719,7 +6708,7 @@
           <t>Beaumont Cherry Valley Recreation &amp; Park District</t>
         </is>
       </c>
-      <c r="D41" s="2" t="n">
+      <c r="D41" s="1" t="n">
         <v>45563</v>
       </c>
       <c r="E41" t="inlineStr">
@@ -6754,7 +6743,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M41" s="2" t="n">
+      <c r="M41" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N41" t="inlineStr"/>
@@ -6773,7 +6762,7 @@
           <t>Alpine Water Users Association</t>
         </is>
       </c>
-      <c r="D42" s="2" t="n">
+      <c r="D42" s="1" t="n">
         <v>46388</v>
       </c>
       <c r="E42" t="inlineStr">
@@ -6808,7 +6797,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M42" s="2" t="n">
+      <c r="M42" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N42" t="inlineStr"/>
@@ -6864,7 +6853,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M43" s="2" t="n">
+      <c r="M43" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N43" t="inlineStr"/>
@@ -6883,7 +6872,7 @@
           <t>Continental Recycling</t>
         </is>
       </c>
-      <c r="D44" s="2" t="n">
+      <c r="D44" s="1" t="n">
         <v>46477</v>
       </c>
       <c r="E44" t="inlineStr">
@@ -6918,7 +6907,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M44" s="2" t="n">
+      <c r="M44" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N44" t="inlineStr"/>
@@ -6937,7 +6926,7 @@
           <t>Discovery Eye Foundation</t>
         </is>
       </c>
-      <c r="D45" s="2" t="n">
+      <c r="D45" s="1" t="n">
         <v>46446</v>
       </c>
       <c r="E45" t="inlineStr">
@@ -6972,7 +6961,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M45" s="2" t="n">
+      <c r="M45" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N45" t="inlineStr"/>
@@ -7007,7 +6996,7 @@
           <t>Dobler Law Group</t>
         </is>
       </c>
-      <c r="D47" s="2" t="n">
+      <c r="D47" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="E47" t="inlineStr">
@@ -7042,7 +7031,7 @@
           <t>Offboarding Phase</t>
         </is>
       </c>
-      <c r="M47" s="2" t="n">
+      <c r="M47" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N47" t="inlineStr"/>
@@ -7098,7 +7087,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M48" s="2" t="n">
+      <c r="M48" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N48" t="inlineStr"/>
@@ -7117,7 +7106,7 @@
           <t>Genesis Supreme &amp; PCW</t>
         </is>
       </c>
-      <c r="D49" s="2" t="n">
+      <c r="D49" s="1" t="n">
         <v>46903</v>
       </c>
       <c r="E49" t="inlineStr">
@@ -7152,7 +7141,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M49" s="2" t="n">
+      <c r="M49" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N49" t="inlineStr"/>
@@ -7208,7 +7197,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M50" s="2" t="n">
+      <c r="M50" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N50" t="inlineStr"/>
@@ -7244,7 +7233,7 @@
       </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
-      <c r="M51" s="2" t="n">
+      <c r="M51" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N51" t="inlineStr"/>
@@ -7263,7 +7252,7 @@
           <t>Larry Jacinto Construction</t>
         </is>
       </c>
-      <c r="D52" s="2" t="n">
+      <c r="D52" s="1" t="n">
         <v>46387</v>
       </c>
       <c r="E52" t="inlineStr">
@@ -7298,7 +7287,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M52" s="2" t="n">
+      <c r="M52" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N52" t="inlineStr"/>
@@ -7317,7 +7306,7 @@
           <t>Lift to Rise</t>
         </is>
       </c>
-      <c r="D53" s="2" t="n">
+      <c r="D53" s="1" t="n">
         <v>45748</v>
       </c>
       <c r="E53" t="inlineStr">
@@ -7352,7 +7341,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M53" s="2" t="n">
+      <c r="M53" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N53" t="inlineStr"/>
@@ -7371,7 +7360,7 @@
           <t>Loma Linda University</t>
         </is>
       </c>
-      <c r="D54" s="2" t="n">
+      <c r="D54" s="1" t="n">
         <v>46904</v>
       </c>
       <c r="E54" t="inlineStr">
@@ -7406,7 +7395,7 @@
           <t xml:space="preserve">Completed </t>
         </is>
       </c>
-      <c r="M54" s="2" t="n">
+      <c r="M54" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N54" t="inlineStr"/>
@@ -7454,7 +7443,7 @@
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
-      <c r="M55" s="2" t="n">
+      <c r="M55" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N55" t="inlineStr"/>
@@ -7473,7 +7462,7 @@
           <t>Open Gym Partner</t>
         </is>
       </c>
-      <c r="D56" s="2" t="n">
+      <c r="D56" s="1" t="n">
         <v>46538</v>
       </c>
       <c r="E56" t="inlineStr">
@@ -7508,7 +7497,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M56" s="2" t="n">
+      <c r="M56" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N56" t="inlineStr"/>
@@ -7527,7 +7516,7 @@
           <t>Riverside County Childcare Consortium</t>
         </is>
       </c>
-      <c r="D57" s="2" t="n">
+      <c r="D57" s="1" t="n">
         <v>46811</v>
       </c>
       <c r="E57" t="inlineStr">
@@ -7562,7 +7551,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M57" s="2" t="n">
+      <c r="M57" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N57" t="inlineStr"/>
@@ -7581,7 +7570,7 @@
           <t>Industry Business Council</t>
         </is>
       </c>
-      <c r="D58" s="2" t="n">
+      <c r="D58" s="1" t="n">
         <v>46965</v>
       </c>
       <c r="E58" t="inlineStr">
@@ -7616,7 +7605,7 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="M58" s="2" t="n">
+      <c r="M58" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N58" t="inlineStr"/>
@@ -7684,7 +7673,7 @@
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
-      <c r="M61" s="2" t="n">
+      <c r="M61" s="1" t="n">
         <v>46006</v>
       </c>
       <c r="N61" t="inlineStr"/>
@@ -7732,58 +7721,58 @@
       <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>CHAMP</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Champion Lumber</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Month To Month</t>
         </is>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" t="n">
         <v>1300</v>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Shaun Alfonso</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Unnamed: 6</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Unnamed: 7</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Unnamed: 8</t>
         </is>
       </c>
-      <c r="J3" s="1" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>11/31/25</t>
         </is>
       </c>
-      <c r="K3" s="1" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Unnamed: 10</t>
         </is>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="L3" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7809,7 +7798,7 @@
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" s="2" t="n">
+      <c r="L4" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7835,7 +7824,7 @@
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" s="2" t="n">
+      <c r="L5" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7861,7 +7850,7 @@
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" s="2" t="n">
+      <c r="L6" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7887,7 +7876,7 @@
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" s="2" t="n">
+      <c r="L7" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7913,7 +7902,7 @@
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" s="2" t="n">
+      <c r="L8" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7939,7 +7928,7 @@
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" s="2" t="n">
+      <c r="L9" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -7997,7 +7986,7 @@
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" s="2" t="n">
+      <c r="L12" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8023,7 +8012,7 @@
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" s="2" t="n">
+      <c r="L13" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8049,7 +8038,7 @@
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" s="2" t="n">
+      <c r="L14" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8067,7 +8056,7 @@
           <t>Lester &amp; Cantrell</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="1" t="n">
         <v>46387</v>
       </c>
       <c r="E15" t="n">
@@ -8083,7 +8072,7 @@
         </is>
       </c>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" s="2" t="n">
+      <c r="L15" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8139,7 +8128,7 @@
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" s="2" t="n">
+      <c r="L18" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8163,7 +8152,7 @@
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" s="2" t="n">
+      <c r="L19" s="1" t="n">
         <v>46006</v>
       </c>
     </row>
@@ -8185,7 +8174,7 @@
       <c r="A1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>vCIO Alingment Answers.docx</t>
         </is>
@@ -8373,37 +8362,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Support Description (Per Unit Per Month)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Unit Pricing</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Current MRC</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Current Qty.</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Applied Discounts</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Current (TrueUP) MRC</t>
         </is>

</xml_diff>

<commit_message>
Dashboard edit: COV in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -695,11 +695,13 @@
           <t>City of Covina</t>
         </is>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>46965</v>
       </c>
-      <c r="D4" t="n">
-        <v>18000</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>18000.0</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -724,29 +726,37 @@
           <t>July- June</t>
         </is>
       </c>
-      <c r="J4" s="1" t="n">
-        <v>46070</v>
-      </c>
-      <c r="K4" t="n">
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-02-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="K4" t="b">
         <v>1</v>
       </c>
-      <c r="L4" s="1" t="n">
-        <v>46072</v>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-02-19 00:00:00</t>
+        </is>
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="n">
+      <c r="R4" t="b">
         <v>1</v>
       </c>
-      <c r="S4" t="n">
-        <v>1</v>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/7jJfr4GR3GrVg4CqCg77Gc8xJh75mFgJPpM3Xcx1?view=grid</t>
+        </is>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
+      <c r="V4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -829,13 +839,11 @@
           <t>City of Duvall</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="1" t="n">
         <v>46074</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>21121.0</t>
-        </is>
+      <c r="D6" t="n">
+        <v>21121</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -857,7 +865,7 @@
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="b">
+      <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -870,7 +878,7 @@
       </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="b">
+      <c r="R6" t="n">
         <v>1</v>
       </c>
       <c r="S6" t="inlineStr">
@@ -880,7 +888,7 @@
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="b">
+      <c r="V6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard edit: MON in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -695,13 +695,11 @@
           <t>City of Covina</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="1" t="n">
         <v>46965</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>18000.0</t>
-        </is>
+      <c r="D4" t="n">
+        <v>18000</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -731,7 +729,7 @@
           <t>2026-02-17 00:00:00</t>
         </is>
       </c>
-      <c r="K4" t="b">
+      <c r="K4" t="n">
         <v>1</v>
       </c>
       <c r="L4" t="inlineStr">
@@ -744,7 +742,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="b">
+      <c r="R4" t="n">
         <v>1</v>
       </c>
       <c r="S4" t="inlineStr">
@@ -754,7 +752,7 @@
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="b">
+      <c r="V4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1043,11 +1041,13 @@
           <t>City of Monrovia</t>
         </is>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="2" t="n">
         <v>47664</v>
       </c>
-      <c r="D9" t="n">
-        <v>36156</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>36156.0</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1068,14 +1068,18 @@
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="1" t="n">
-        <v>46077</v>
-      </c>
-      <c r="K9" t="n">
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-02-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="K9" t="b">
         <v>1</v>
       </c>
-      <c r="L9" s="1" t="n">
-        <v>46078</v>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-02-25 00:00:00</t>
+        </is>
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -1090,15 +1094,19 @@
           <t>Local Backup (CB)</t>
         </is>
       </c>
-      <c r="R9" t="n">
+      <c r="R9" t="b">
         <v>1</v>
       </c>
-      <c r="S9" t="n">
-        <v>1</v>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/4XG65x3p4RwQgmQWH3q4Jx6rrf2rhJfvPgwJ9w51?view=grid</t>
+        </is>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
+      <c r="V9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: CSF in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -1041,13 +1041,11 @@
           <t>City of Monrovia</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="1" t="n">
         <v>47664</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>36156.0</t>
-        </is>
+      <c r="D9" t="n">
+        <v>36156</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1073,7 +1071,7 @@
           <t>2026-02-24 00:00:00</t>
         </is>
       </c>
-      <c r="K9" t="b">
+      <c r="K9" t="n">
         <v>1</v>
       </c>
       <c r="L9" t="inlineStr">
@@ -1094,7 +1092,7 @@
           <t>Local Backup (CB)</t>
         </is>
       </c>
-      <c r="R9" t="b">
+      <c r="R9" t="n">
         <v>1</v>
       </c>
       <c r="S9" t="inlineStr">
@@ -1104,7 +1102,7 @@
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
-      <c r="V9" t="b">
+      <c r="V9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1183,11 +1181,13 @@
           <t>City of San Fernando</t>
         </is>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="2" t="n">
         <v>46326</v>
       </c>
-      <c r="D11" t="n">
-        <v>17154</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>17154.0</t>
+        </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1209,8 +1209,8 @@
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="n">
-        <v>0</v>
+      <c r="K11" t="b">
+        <v>1</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
@@ -1222,15 +1222,19 @@
       </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="n">
+      <c r="R11" t="b">
         <v>1</v>
       </c>
-      <c r="S11" t="n">
-        <v>1</v>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/H8fm5w2CPG33cjhfw3QcFp7x3FgqpqcRHWm48221?view=grid</t>
+        </is>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
+      <c r="V11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: RPV in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -1117,11 +1117,13 @@
           <t>City of Ranchos Palos Verdes</t>
         </is>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="2" t="n">
         <v>46559</v>
       </c>
-      <c r="D10" t="n">
-        <v>14986</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>14986.0</t>
+        </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1143,7 +1145,7 @@
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="n">
+      <c r="K10" t="b">
         <v>0</v>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1160,15 +1162,19 @@
           <t>Local Backup/VEEAM (CB)</t>
         </is>
       </c>
-      <c r="R10" t="n">
+      <c r="R10" t="b">
         <v>1</v>
       </c>
-      <c r="S10" t="n">
-        <v>1</v>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/VmCFPV3Q6P3Hmvjhjq5cqWqJXXJ3FRX2vWvRPhQ1?view=grid</t>
+        </is>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
+      <c r="V10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1181,13 +1187,11 @@
           <t>City of San Fernando</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="1" t="n">
         <v>46326</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>17154.0</t>
-        </is>
+      <c r="D11" t="n">
+        <v>17154</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1213,7 +1217,7 @@
           <t>04/01/2026</t>
         </is>
       </c>
-      <c r="K11" t="b">
+      <c r="K11" t="n">
         <v>1</v>
       </c>
       <c r="L11" t="inlineStr">
@@ -1230,7 +1234,7 @@
       </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="b">
+      <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="inlineStr">
@@ -1240,7 +1244,7 @@
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
-      <c r="V11" t="b">
+      <c r="V11" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard edit: COI in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -973,11 +973,13 @@
           <t>City of Industry</t>
         </is>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="2" t="n">
         <v>46326</v>
       </c>
-      <c r="D8" t="n">
-        <v>22800</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>22800.0</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -999,7 +1001,7 @@
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="n">
+      <c r="K8" t="b">
         <v>0</v>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1020,15 +1022,19 @@
           <t>VEEAM (CB)</t>
         </is>
       </c>
-      <c r="R8" t="n">
+      <c r="R8" t="b">
         <v>1</v>
       </c>
-      <c r="S8" t="n">
-        <v>1</v>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/WrPjV776cqwRqC9G4Cjv6jjW43Vg8jf8xcM47Qq1?view=grid</t>
+        </is>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
+      <c r="V8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1117,13 +1123,11 @@
           <t>City of Ranchos Palos Verdes</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="1" t="n">
         <v>46559</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>14986.0</t>
-        </is>
+      <c r="D10" t="n">
+        <v>14986</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1145,7 +1149,7 @@
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="b">
+      <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1162,7 +1166,7 @@
           <t>Local Backup/VEEAM (CB)</t>
         </is>
       </c>
-      <c r="R10" t="b">
+      <c r="R10" t="n">
         <v>1</v>
       </c>
       <c r="S10" t="inlineStr">
@@ -1172,7 +1176,7 @@
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="b">
+      <c r="V10" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard edit: COJK in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -623,11 +623,13 @@
           <t>Christensen, O'Connor, Johnson, Kindness</t>
         </is>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>46554</v>
       </c>
-      <c r="D3" t="n">
-        <v>30561</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>30561.0</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -648,14 +650,18 @@
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="1" t="n">
-        <v>46044</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-01-22 00:00:00</t>
+        </is>
+      </c>
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-01-22 00:00:00</t>
+        </is>
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -674,15 +680,19 @@
           <t>Azure (NC)</t>
         </is>
       </c>
-      <c r="R3" t="n">
+      <c r="R3" t="b">
         <v>1</v>
       </c>
-      <c r="S3" t="n">
-        <v>1</v>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/742CXRmjRXrjPHpJqG338GvqCcf4GgGFVcxx8cG1?view=grid</t>
+        </is>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
+      <c r="V3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -973,13 +983,11 @@
           <t>City of Industry</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="1" t="n">
         <v>46326</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>22800.0</t>
-        </is>
+      <c r="D8" t="n">
+        <v>22800</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1001,7 +1009,7 @@
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="b">
+      <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1022,7 +1030,7 @@
           <t>VEEAM (CB)</t>
         </is>
       </c>
-      <c r="R8" t="b">
+      <c r="R8" t="n">
         <v>1</v>
       </c>
       <c r="S8" t="inlineStr">
@@ -1032,7 +1040,7 @@
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="b">
+      <c r="V8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard edit: COG in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -623,13 +623,11 @@
           <t>Christensen, O'Connor, Johnson, Kindness</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="1" t="n">
         <v>46554</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>30561.0</t>
-        </is>
+      <c r="D3" t="n">
+        <v>30561</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -655,7 +653,7 @@
           <t>2026-01-22 00:00:00</t>
         </is>
       </c>
-      <c r="K3" t="b">
+      <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="inlineStr">
@@ -680,7 +678,7 @@
           <t>Azure (NC)</t>
         </is>
       </c>
-      <c r="R3" t="b">
+      <c r="R3" t="n">
         <v>1</v>
       </c>
       <c r="S3" t="inlineStr">
@@ -690,7 +688,7 @@
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
-      <c r="V3" t="b">
+      <c r="V3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -911,11 +909,13 @@
           <t>City of Goleta</t>
         </is>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="2" t="n">
         <v>46568</v>
       </c>
-      <c r="D7" t="n">
-        <v>26500</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>26500.0</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -940,14 +940,18 @@
           <t>July-June</t>
         </is>
       </c>
-      <c r="J7" s="1" t="n">
-        <v>46043</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="1" t="n">
-        <v>46044</v>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-01-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-01-22 00:00:00</t>
+        </is>
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -962,15 +966,19 @@
           <t>Datto Endpoint Backup (CB)</t>
         </is>
       </c>
-      <c r="R7" t="n">
+      <c r="R7" t="b">
         <v>1</v>
       </c>
-      <c r="S7" t="n">
-        <v>1</v>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/CM5P2VxFQ5hqPr3R22cgFCc3wC793Cpjgx3QjVg1?view=grid</t>
+        </is>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
+      <c r="V7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: DWA in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -909,13 +909,11 @@
           <t>City of Goleta</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="1" t="n">
         <v>46568</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>26500.0</t>
-        </is>
+      <c r="D7" t="n">
+        <v>26500</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -945,7 +943,7 @@
           <t>2026-01-21 00:00:00</t>
         </is>
       </c>
-      <c r="K7" t="b">
+      <c r="K7" t="n">
         <v>0</v>
       </c>
       <c r="L7" t="inlineStr">
@@ -966,7 +964,7 @@
           <t>Datto Endpoint Backup (CB)</t>
         </is>
       </c>
-      <c r="R7" t="b">
+      <c r="R7" t="n">
         <v>1</v>
       </c>
       <c r="S7" t="inlineStr">
@@ -976,7 +974,7 @@
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="b">
+      <c r="V7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1555,11 +1553,13 @@
           <t>Desert Water Agency</t>
         </is>
       </c>
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="2" t="n">
         <v>45530</v>
       </c>
-      <c r="D16" t="n">
-        <v>9120</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>9120.0</t>
+        </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1580,14 +1580,18 @@
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="1" t="n">
-        <v>46083</v>
-      </c>
-      <c r="K16" t="n">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-03-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="K16" t="b">
         <v>1</v>
       </c>
-      <c r="L16" s="1" t="n">
-        <v>46085</v>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-03-04 00:00:00</t>
+        </is>
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
@@ -1602,15 +1606,19 @@
           <t>Local Backup (CB)</t>
         </is>
       </c>
-      <c r="R16" t="n">
+      <c r="R16" t="b">
         <v>1</v>
       </c>
-      <c r="S16" t="n">
-        <v>1</v>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/M8Ch5J6FQjm29rjfc3XMMrhm2H2fRCG8v3QX5xV1?view=grid</t>
+        </is>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+      <c r="V16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: ACC in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -1553,13 +1553,11 @@
           <t>Desert Water Agency</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="1" t="n">
         <v>45530</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>9120.0</t>
-        </is>
+      <c r="D16" t="n">
+        <v>9120</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1585,7 +1583,7 @@
           <t>2026-03-02 00:00:00</t>
         </is>
       </c>
-      <c r="K16" t="b">
+      <c r="K16" t="n">
         <v>1</v>
       </c>
       <c r="L16" t="inlineStr">
@@ -1606,7 +1604,7 @@
           <t>Local Backup (CB)</t>
         </is>
       </c>
-      <c r="R16" t="b">
+      <c r="R16" t="n">
         <v>1</v>
       </c>
       <c r="S16" t="inlineStr">
@@ -1616,7 +1614,7 @@
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="b">
+      <c r="V16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1631,11 +1629,13 @@
           <t>Adams Campbell Construction</t>
         </is>
       </c>
-      <c r="C17" s="1" t="n">
+      <c r="C17" s="2" t="n">
         <v>46419</v>
       </c>
-      <c r="D17" t="n">
-        <v>4659</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>4659.0</t>
+        </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="n">
+      <c r="K17" t="b">
         <v>0</v>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -1674,15 +1674,19 @@
           <t>Local Backup (CB)</t>
         </is>
       </c>
-      <c r="R17" t="n">
+      <c r="R17" t="b">
         <v>1</v>
       </c>
-      <c r="S17" t="n">
-        <v>1</v>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/hrhcx2GJx4MW293cmr4jfw7JjCCrqV8C95pr8Fr1?view=grid</t>
+        </is>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
+      <c r="V17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard edit: HESP in Customer status
</commit_message>
<xml_diff>
--- a/Customer Contract and MRC Tracking.xlsx
+++ b/Customer Contract and MRC Tracking.xlsx
@@ -2033,13 +2033,11 @@
           <t>CMSD</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n">
+      <c r="C23" s="1" t="n">
         <v>46203</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>5730.0</t>
-        </is>
+      <c r="D23" t="n">
+        <v>5730</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2065,7 +2063,7 @@
           <t>2026-03-04 00:00:00</t>
         </is>
       </c>
-      <c r="K23" t="b">
+      <c r="K23" t="n">
         <v>1</v>
       </c>
       <c r="L23" t="inlineStr">
@@ -2082,7 +2080,7 @@
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="b">
+      <c r="R23" t="n">
         <v>1</v>
       </c>
       <c r="S23" t="inlineStr">
@@ -2092,7 +2090,7 @@
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="b">
+      <c r="V23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2107,11 +2105,13 @@
           <t>Hesperia Recreation and Park District</t>
         </is>
       </c>
-      <c r="C24" s="1" t="n">
+      <c r="C24" s="2" t="n">
         <v>45303</v>
       </c>
-      <c r="D24" t="n">
-        <v>3967</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>3967.0</t>
+        </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" t="n">
+      <c r="K24" t="b">
         <v>0</v>
       </c>
       <c r="L24" t="inlineStr"/>
@@ -2150,15 +2150,19 @@
           <t>NEEDS NAS URGENTLY Local Backup/VEEAM (CB)</t>
         </is>
       </c>
-      <c r="R24" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" t="n">
-        <v>1</v>
+      <c r="R24" t="b">
+        <v>0</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>https://app.smartsheet.com/sheets/Wp93WJ7rjJR9xGr54pGfQ5g6XV3vhWPM943xqc81?view=grid</t>
+        </is>
       </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
+      <c r="V24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>